<commit_message>
Update hotel pricing data and change history
</commit_message>
<xml_diff>
--- a/change_history.xlsx
+++ b/change_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,22 +458,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Single Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -483,12 +483,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -496,66 +496,62 @@
           <t>Twin Room</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Double Room</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Double Room</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -565,22 +561,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -600,12 +596,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,17 +621,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -650,130 +646,138 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>Triple Room</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>Single Room</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>Triple Room</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>Triple Room</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -782,43 +786,43 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -828,22 +832,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -851,20 +855,24 @@
           <t>Twin Room</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -872,20 +880,24 @@
           <t>Twin Room</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -895,464 +907,36 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Single Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
         <v>8</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-03-30</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-03-31</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-03-31</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-04-18</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026-04-19</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2026-11-22</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
입력 속도 복원: 2-retry 검증 모드 + SLEEP_SCALE 0.5로 변경
- set_input_value()를 send_keys + 값 검증 + JS fallback 로직으로 복원
- SLEEP_SCALE을 0.35에서 0.5로 조정 (안전한 중간 속도)
- Trip.com 15-20% 로직 및 마감일 스킵 기능 유지
</commit_message>
<xml_diff>
--- a/change_history.xlsx
+++ b/change_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,12 +458,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -473,160 +473,170 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Triple Room</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Double Room</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Twin Room</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Double Room</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Twin Room</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>5</v>
-      </c>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -636,307 +646,36 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Twin Room</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Excel history and highlight data
</commit_message>
<xml_diff>
--- a/change_history.xlsx
+++ b/change_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,28 +458,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Single Room</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>Triple Room</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -492,120 +496,116 @@
           <t>Single Room</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
-        <v>4</v>
-      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Triple Room</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>Single Room</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
-      </c>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Triple Room</t>
+          <t>Twin Room</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,12 +625,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -640,22 +640,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -665,22 +665,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>9</v>
-      </c>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -690,47 +688,45 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Twin Room</t>
+          <t>Single Room</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>6</v>
-      </c>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -740,7 +736,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -750,12 +746,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -773,12 +769,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -788,7 +784,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -796,12 +792,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -815,6 +811,100 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Double Room</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Double Room</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Double Room</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Double Room</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>